<commit_message>
Cambio en entregable 2
</commit_message>
<xml_diff>
--- a/DJF/FTs/UAH_ASW SVT_TestProcedures.xlsx
+++ b/DJF/FTs/UAH_ASW SVT_TestProcedures.xlsx
@@ -23,12 +23,11 @@
     <sheet name="FT_UAH_ASW_SERV_128-0200" sheetId="8" r:id="rId9"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="137">
   <si>
     <t>Doc. No.:</t>
   </si>
@@ -464,6 +463,9 @@
       </rPr>
       <t>TODO</t>
     </r>
+  </si>
+  <si>
+    <t>PMONID=0, PID=15, value=5, limit=1, prev status Unchecked, current status Within Limits</t>
   </si>
 </sst>
 </file>
@@ -843,7 +845,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1045,6 +1047,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9790,12 +9793,16 @@
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="12.75" customHeight="1">
+    <row r="45" spans="1:5" ht="76.2" customHeight="1">
       <c r="A45" s="72"/>
       <c r="B45" s="108"/>
       <c r="C45" s="85"/>
-      <c r="D45" s="85"/>
-      <c r="E45" s="75"/>
+      <c r="D45" s="109" t="s">
+        <v>129</v>
+      </c>
+      <c r="E45" s="97" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="46" spans="1:5" ht="12.75" customHeight="1">
       <c r="A46" s="86" t="s">

</xml_diff>